<commit_message>
added new tab to give clear info
</commit_message>
<xml_diff>
--- a/public/Halt Claims Scenarios.xlsx
+++ b/public/Halt Claims Scenarios.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susmitamadineni/Projects.nosync/claims-sum/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC15DA5-24D0-1C4A-8AA3-B84A4751530C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55444784-8319-E44A-92D2-E2F21070788F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{578A4F4A-DD6A-DF4D-B5F9-009FA3AD108E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="64">
   <si>
     <t>CATEGORY</t>
   </si>
@@ -68,12 +68,6 @@
     <t>REASON_CODE</t>
   </si>
   <si>
-    <t>Member Search - Prepopulated Search criteria</t>
-  </si>
-  <si>
-    <t>Employer group Search - Prepopulated Search criteria</t>
-  </si>
-  <si>
     <t>Member Match Rules</t>
   </si>
   <si>
@@ -131,42 +125,6 @@
     <t>HALT_ENROLL</t>
   </si>
   <si>
-    <t>Focused and Highlighted - Service Date; Network</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network; Last Name; First Name</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network; First Name; Date Of Birth</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network; Last Name; Date Of Birth</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; Last Name; First Name</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; Last Name</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; Date Of Birth; Gender</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; Gender</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; First Name; Date Of Birth</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Service Date; Network;Insured ID; First Name; Gender</t>
-  </si>
-  <si>
-    <t>Highlighted - Policy#/Alias; Network</t>
-  </si>
-  <si>
     <t>Employer group Policy Match Results</t>
   </si>
   <si>
@@ -212,22 +170,67 @@
     <t>DISCREPANCY_BETWN_PARENT_CODES</t>
   </si>
   <si>
-    <t>Highlighted - Service Date; Network</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Network; Group Name/Alias</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Network; Policy#/Alias</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Network; Parent Code Desc/Alias</t>
-  </si>
-  <si>
-    <t>Focused and Highlighted - Network; Client Code</t>
-  </si>
-  <si>
-    <t>Highlighted - Network; Policy#/Alias</t>
+    <t>Focused MFE</t>
+  </si>
+  <si>
+    <t>Member Search</t>
+  </si>
+  <si>
+    <t>Service Date; Network</t>
+  </si>
+  <si>
+    <t>Employer group Search</t>
+  </si>
+  <si>
+    <t>Service Date; Network; Last Name; First Name</t>
+  </si>
+  <si>
+    <t>Service Date; Network; First Name; Date Of Birth</t>
+  </si>
+  <si>
+    <t>Service Date; Network; Last Name; Date Of Birth</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; Last Name; First Name</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; Last Name</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; Date Of Birth; Gender</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; Gender</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; First Name; Gender</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID; First Name; Date Of Birth</t>
+  </si>
+  <si>
+    <t>Service Date; Network;Insured ID</t>
+  </si>
+  <si>
+    <t>Network; Group Name/Alias</t>
+  </si>
+  <si>
+    <t>Network; Policy#/Alias</t>
+  </si>
+  <si>
+    <t>Network; Parent Code Desc/Alias</t>
+  </si>
+  <si>
+    <t>Network; Client Code</t>
+  </si>
+  <si>
+    <t>Policy#/Alias; Network</t>
+  </si>
+  <si>
+    <t>Member Search MFE - Prepopulated Search criteria - Highlighted fields</t>
+  </si>
+  <si>
+    <t>Employer group Search MFE - Prepopulated Search criteria - Highlighted fields</t>
   </si>
 </sst>
 </file>
@@ -682,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92307686-27A4-DC4D-B5C8-FA7B30A50B51}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -693,14 +696,15 @@
     <col min="7" max="7" width="13" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="39.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="45" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.83203125" style="1"/>
+    <col min="10" max="10" width="13.83203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="39.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="45" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -711,9 +715,10 @@
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="K1" s="5"/>
+      <c r="L1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -742,21 +747,24 @@
         <v>8</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="K2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="B3" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2">
         <v>685</v>
@@ -765,33 +773,36 @@
         <v>1301</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2">
         <v>685</v>
@@ -800,33 +811,36 @@
         <v>1401</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2">
         <v>685</v>
@@ -835,33 +849,36 @@
         <v>1402</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2">
         <v>685</v>
@@ -870,33 +887,36 @@
         <v>1403</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2">
         <v>685</v>
@@ -905,33 +925,36 @@
         <v>1501</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" s="2">
         <v>685</v>
@@ -940,33 +963,36 @@
         <v>1502</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2">
         <v>685</v>
@@ -975,33 +1001,36 @@
         <v>1503</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2">
         <v>685</v>
@@ -1010,33 +1039,36 @@
         <v>1504</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2">
         <v>685</v>
@@ -1045,33 +1077,36 @@
         <v>1505</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D12" s="2">
         <v>685</v>
@@ -1080,33 +1115,36 @@
         <v>1506</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="J12" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D13" s="2">
         <v>685</v>
@@ -1115,25 +1153,28 @@
         <v>1507</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1145,10 +1186,11 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1159,9 +1201,10 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="6"/>
-    </row>
-    <row r="16" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="K15" s="5"/>
+      <c r="L15" s="6"/>
+    </row>
+    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -1190,21 +1233,24 @@
         <v>8</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D17" s="2">
         <v>685</v>
@@ -1213,33 +1259,36 @@
         <v>3301</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J17" s="2" t="s">
+      <c r="L17" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D18" s="2">
         <v>685</v>
@@ -1248,33 +1297,36 @@
         <v>3401</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D19" s="2">
         <v>685</v>
@@ -1283,33 +1335,36 @@
         <v>3501</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D20" s="2">
         <v>685</v>
@@ -1318,33 +1373,36 @@
         <v>3601</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2">
         <v>685</v>
@@ -1353,25 +1411,28 @@
         <v>3701</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1383,10 +1444,11 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1397,9 +1459,10 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
-      <c r="K23" s="6"/>
-    </row>
-    <row r="24" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="K23" s="5"/>
+      <c r="L23" s="6"/>
+    </row>
+    <row r="24" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>0</v>
       </c>
@@ -1428,21 +1491,24 @@
         <v>8</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D25" s="2">
         <v>685</v>
@@ -1451,33 +1517,36 @@
         <v>7001</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D26" s="2">
         <v>685</v>
@@ -1486,33 +1555,36 @@
         <v>7002</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D27" s="2">
         <v>685</v>
@@ -1521,25 +1593,28 @@
         <v>7003</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1551,8 +1626,9 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1564,8 +1640,9 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1577,8 +1654,9 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1590,8 +1668,9 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1603,8 +1682,9 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" s="2"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1616,8 +1696,9 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" s="2"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1629,8 +1710,9 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" s="2"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1642,12 +1724,13 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A23:L23"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>